<commit_message>
Refactor index.html and remove unused Excel files
</commit_message>
<xml_diff>
--- a/Hasil_Ekstraksi/Hasil_Prediksi_RandomForest.xlsx
+++ b/Hasil_Ekstraksi/Hasil_Prediksi_RandomForest.xlsx
@@ -10,6 +10,7 @@
     <sheet name="1_Prediksi_RandomForest" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2_Tabel_Metrik_Evaluasi" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3_Scatter_Plot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4_Histogram_ExG" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -245,6 +246,36 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5905500" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1333,4 +1364,33 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DISTRIBUSI NILAI EXCESS GREEN (ExG) - 16 SAMPEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Buat lihat sebaran nilai ExG antar sampel, bukan buat bandingin aktual vs prediksi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>